<commit_message>
Update and allow for publish?
</commit_message>
<xml_diff>
--- a/Python/FinishTemplate.xlsx
+++ b/Python/FinishTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\source\repos\CycleScoresWeb\Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CAF1AA2-DE9D-45B6-A83E-52870BC629DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14CD2480-C54D-447C-AD5A-858F2C015C5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15585" yWindow="2610" windowWidth="26580" windowHeight="18915" xr2:uid="{99C8F65C-2FC9-4F92-82E2-8DAB5ADF2049}"/>
+    <workbookView xWindow="2070" yWindow="4155" windowWidth="26505" windowHeight="11490" xr2:uid="{99C8F65C-2FC9-4F92-82E2-8DAB5ADF2049}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="55">
   <si>
     <t>Event</t>
   </si>
@@ -71,12 +71,6 @@
     <t>CommuniqueType</t>
   </si>
   <si>
-    <t>Women Elite - Omnium Scratch</t>
-  </si>
-  <si>
-    <t>7.5km / 17 laps</t>
-  </si>
-  <si>
     <t>Bib</t>
   </si>
   <si>
@@ -86,63 +80,12 @@
     <t>Nation</t>
   </si>
   <si>
-    <t>WINTHER OLSEN Amalie</t>
-  </si>
-  <si>
-    <t>JESSETT Miriam</t>
-  </si>
-  <si>
-    <t>HOMER Gabriella</t>
-  </si>
-  <si>
-    <t>SODEN Nicola</t>
-  </si>
-  <si>
-    <t>HALSEY Sasha</t>
-  </si>
-  <si>
-    <t>WATKINSON Dannielle</t>
-  </si>
-  <si>
-    <t>BOOTHMAN Erin</t>
-  </si>
-  <si>
-    <t>CADMAN Hannah</t>
-  </si>
-  <si>
-    <t>DEN</t>
-  </si>
-  <si>
     <t>GBR</t>
   </si>
   <si>
     <t>IRL</t>
   </si>
   <si>
-    <t>SELVA Francesca</t>
-  </si>
-  <si>
-    <t>NELSON Lucy</t>
-  </si>
-  <si>
-    <t>MAC HALE Keela</t>
-  </si>
-  <si>
-    <t>CORNELIUS Jasmine</t>
-  </si>
-  <si>
-    <t>FERGUSON Cat</t>
-  </si>
-  <si>
-    <t>BARNWELL Ella</t>
-  </si>
-  <si>
-    <t>GLOVER Lucy</t>
-  </si>
-  <si>
-    <t>ITA</t>
-  </si>
-  <si>
     <t>Rank</t>
   </si>
   <si>
@@ -152,10 +95,115 @@
     <t>Result</t>
   </si>
   <si>
-    <t>011</t>
-  </si>
-  <si>
-    <t>DNF</t>
+    <t>032</t>
+  </si>
+  <si>
+    <t>Men Elite - Elimination Race</t>
+  </si>
+  <si>
+    <t>COL</t>
+  </si>
+  <si>
+    <t>SWE</t>
+  </si>
+  <si>
+    <t>LAT</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>LTU</t>
+  </si>
+  <si>
+    <t>BRIGGS Alec</t>
+  </si>
+  <si>
+    <t>VAUGHAN Jacob</t>
+  </si>
+  <si>
+    <t>AMBROSE PARISH James</t>
+  </si>
+  <si>
+    <t>PERRETT William</t>
+  </si>
+  <si>
+    <t>HOLT Joe</t>
+  </si>
+  <si>
+    <t>CADAVID RIVERA Santiago Isaac</t>
+  </si>
+  <si>
+    <t>JOHANSSON Gustav</t>
+  </si>
+  <si>
+    <t>BELTON OWEN Dylan</t>
+  </si>
+  <si>
+    <t>LONGSTAFF Frank</t>
+  </si>
+  <si>
+    <t>BREARLEY David</t>
+  </si>
+  <si>
+    <t>FOUGO Tiago</t>
+  </si>
+  <si>
+    <t>BRITTON Rhys</t>
+  </si>
+  <si>
+    <t>HARDY Nathan</t>
+  </si>
+  <si>
+    <t>NEMILOSTIVIJS George</t>
+  </si>
+  <si>
+    <t>INNISS Nimai</t>
+  </si>
+  <si>
+    <t>BYRNE Ryan</t>
+  </si>
+  <si>
+    <t>WHITEHOUSE Jack</t>
+  </si>
+  <si>
+    <t>JOHNSON Christopher</t>
+  </si>
+  <si>
+    <t>STEWART Joel</t>
+  </si>
+  <si>
+    <t>TORRIE Timothy</t>
+  </si>
+  <si>
+    <t>PHILLIPS Noah</t>
+  </si>
+  <si>
+    <t>BRINKLEY Andrew</t>
+  </si>
+  <si>
+    <t>BOWIE John</t>
+  </si>
+  <si>
+    <t>MEYER-ELAND Luke</t>
+  </si>
+  <si>
+    <t>DAVIES Euan</t>
+  </si>
+  <si>
+    <t>WARD Tom</t>
+  </si>
+  <si>
+    <t>HARRIS Jonah</t>
+  </si>
+  <si>
+    <t>KAZINEC Viktor</t>
+  </si>
+  <si>
+    <t>DELICAET Len</t>
+  </si>
+  <si>
+    <t>GRIFFIN Ross</t>
   </si>
 </sst>
 </file>
@@ -217,9 +265,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -257,7 +305,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -363,7 +411,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -505,7 +553,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -513,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E69E43A-04DB-4D93-BF53-73900B0B455F}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.5703125" bestFit="1" customWidth="1"/>
@@ -548,7 +596,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -558,7 +606,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -568,7 +616,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -577,9 +625,7 @@
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
     </row>
@@ -610,266 +656,472 @@
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="F10" s="1" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="1">
+      <c r="B11">
         <v>1</v>
       </c>
-      <c r="C11" s="1">
-        <v>5</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>24</v>
+      <c r="C11">
+        <v>40</v>
+      </c>
+      <c r="D11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" t="s">
+        <v>13</v>
       </c>
       <c r="F11" s="1"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="1">
+      <c r="B12">
         <v>2</v>
       </c>
-      <c r="C12" s="1">
-        <v>3</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>24</v>
+      <c r="C12">
+        <v>52</v>
+      </c>
+      <c r="D12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" t="s">
+        <v>13</v>
       </c>
       <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="B13" s="1">
+      <c r="B13">
         <v>3</v>
       </c>
-      <c r="C13" s="1">
-        <v>6</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>24</v>
+      <c r="C13">
+        <v>53</v>
+      </c>
+      <c r="D13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
       </c>
       <c r="F13" s="1"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="1">
+      <c r="B14">
         <v>4</v>
       </c>
-      <c r="C14" s="1">
-        <v>13</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>24</v>
+      <c r="C14">
+        <v>71</v>
+      </c>
+      <c r="D14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" t="s">
+        <v>13</v>
       </c>
       <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="1">
+      <c r="B15">
         <v>5</v>
       </c>
-      <c r="C15" s="1">
-        <v>14</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>24</v>
+      <c r="C15">
+        <v>54</v>
+      </c>
+      <c r="D15" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
       </c>
       <c r="F15" s="1"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="1">
+      <c r="B16">
         <v>6</v>
       </c>
-      <c r="C16" s="1">
-        <v>9</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>24</v>
+      <c r="C16">
+        <v>66</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" t="s">
+        <v>20</v>
       </c>
       <c r="F16" s="1"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="1">
+      <c r="B17">
         <v>7</v>
       </c>
-      <c r="C17" s="1">
-        <v>1</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>23</v>
+      <c r="C17">
+        <v>49</v>
+      </c>
+      <c r="D17" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17" t="s">
+        <v>21</v>
       </c>
       <c r="F17" s="1"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="1">
+      <c r="B18">
         <v>8</v>
       </c>
-      <c r="C18" s="1">
-        <v>8</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>25</v>
+      <c r="C18">
+        <v>45</v>
+      </c>
+      <c r="D18" t="s">
+        <v>32</v>
+      </c>
+      <c r="E18" t="s">
+        <v>13</v>
       </c>
       <c r="F18" s="1"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
-      <c r="B19" s="1">
+      <c r="B19">
         <v>9</v>
       </c>
-      <c r="C19" s="1">
-        <v>7</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E19" s="1" t="s">
+      <c r="C19">
+        <v>47</v>
+      </c>
+      <c r="D19" t="s">
         <v>33</v>
+      </c>
+      <c r="E19" t="s">
+        <v>13</v>
       </c>
       <c r="F19" s="1"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
-      <c r="B20" s="1">
+      <c r="B20">
         <v>10</v>
       </c>
-      <c r="C20" s="1">
-        <v>15</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>24</v>
+      <c r="C20">
+        <v>44</v>
+      </c>
+      <c r="D20" t="s">
+        <v>34</v>
+      </c>
+      <c r="E20" t="s">
+        <v>13</v>
       </c>
       <c r="F20" s="1"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="1">
+      <c r="B21">
         <v>11</v>
       </c>
-      <c r="C21" s="1">
-        <v>4</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>24</v>
+      <c r="C21">
+        <v>67</v>
+      </c>
+      <c r="D21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E21" t="s">
+        <v>13</v>
       </c>
       <c r="F21" s="1"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="1">
+      <c r="B22">
         <v>12</v>
       </c>
-      <c r="C22" s="1">
-        <v>17</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>24</v>
+      <c r="C22">
+        <v>63</v>
+      </c>
+      <c r="D22" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" t="s">
+        <v>13</v>
       </c>
       <c r="F22" s="1"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="1">
-        <v>13</v>
-      </c>
-      <c r="C23" s="1">
-        <v>16</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>24</v>
+      <c r="B23">
+        <v>13</v>
+      </c>
+      <c r="C23">
+        <v>59</v>
+      </c>
+      <c r="D23" t="s">
+        <v>37</v>
+      </c>
+      <c r="E23" t="s">
+        <v>13</v>
       </c>
       <c r="F23" s="1"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
-      <c r="B24" s="1">
+      <c r="B24">
         <v>14</v>
       </c>
-      <c r="C24" s="1">
-        <v>10</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>25</v>
+      <c r="C24">
+        <v>48</v>
+      </c>
+      <c r="D24" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" t="s">
+        <v>22</v>
       </c>
       <c r="F24" s="1"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C25" s="1">
-        <v>32</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>24</v>
+      <c r="B25">
+        <v>15</v>
+      </c>
+      <c r="C25">
+        <v>61</v>
+      </c>
+      <c r="D25" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25" t="s">
+        <v>13</v>
       </c>
       <c r="F25" s="1"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
+      <c r="B26">
+        <v>16</v>
+      </c>
+      <c r="C26">
+        <v>65</v>
+      </c>
+      <c r="D26" t="s">
+        <v>40</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
+      <c r="B27">
+        <v>17</v>
+      </c>
+      <c r="C27">
+        <v>51</v>
+      </c>
+      <c r="D27" t="s">
+        <v>41</v>
+      </c>
+      <c r="E27" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B28">
+        <v>18</v>
+      </c>
+      <c r="C28">
+        <v>43</v>
+      </c>
+      <c r="D28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E28" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B29">
+        <v>19</v>
+      </c>
+      <c r="C29">
+        <v>55</v>
+      </c>
+      <c r="D29" t="s">
+        <v>43</v>
+      </c>
+      <c r="E29" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B30">
+        <v>20</v>
+      </c>
+      <c r="C30">
+        <v>68</v>
+      </c>
+      <c r="D30" t="s">
+        <v>44</v>
+      </c>
+      <c r="E30" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B31">
+        <v>21</v>
+      </c>
+      <c r="C31">
+        <v>62</v>
+      </c>
+      <c r="D31" t="s">
+        <v>45</v>
+      </c>
+      <c r="E31" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B32">
+        <v>22</v>
+      </c>
+      <c r="C32">
+        <v>41</v>
+      </c>
+      <c r="D32" t="s">
+        <v>46</v>
+      </c>
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B33">
+        <v>23</v>
+      </c>
+      <c r="C33">
+        <v>56</v>
+      </c>
+      <c r="D33" t="s">
+        <v>47</v>
+      </c>
+      <c r="E33" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B34">
+        <v>24</v>
+      </c>
+      <c r="C34">
+        <v>58</v>
+      </c>
+      <c r="D34" t="s">
+        <v>48</v>
+      </c>
+      <c r="E34" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B35">
+        <v>25</v>
+      </c>
+      <c r="C35">
+        <v>46</v>
+      </c>
+      <c r="D35" t="s">
+        <v>49</v>
+      </c>
+      <c r="E35" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B36">
+        <v>26</v>
+      </c>
+      <c r="C36">
+        <v>69</v>
+      </c>
+      <c r="D36" t="s">
+        <v>50</v>
+      </c>
+      <c r="E36" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B37">
+        <v>27</v>
+      </c>
+      <c r="C37">
+        <v>57</v>
+      </c>
+      <c r="D37" t="s">
+        <v>51</v>
+      </c>
+      <c r="E37" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B38">
+        <v>28</v>
+      </c>
+      <c r="C38">
+        <v>70</v>
+      </c>
+      <c r="D38" t="s">
+        <v>52</v>
+      </c>
+      <c r="E38" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B39">
+        <v>29</v>
+      </c>
+      <c r="C39">
+        <v>72</v>
+      </c>
+      <c r="D39" t="s">
+        <v>53</v>
+      </c>
+      <c r="E39" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B40">
+        <v>30</v>
+      </c>
+      <c r="C40">
+        <v>64</v>
+      </c>
+      <c r="D40" t="s">
+        <v>54</v>
+      </c>
+      <c r="E40" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B11:F25">

</xml_diff>